<commit_message>
seed_ftl: rantai FTL Normal tuntas end-to-end; loop lebih kebal
FTL beda kontrak dari LTL: tipePengiriman + jenisArmadaId + jumlahArmada
ikut di level shipment (buat_shipment kini menerima `extra`). Pilot
SHP26080010 → FTL6940683725 selesai 4 tahap tanpa ditagih resi, dan
push FCM penugasan terverifikasi ("Anda menerima tugas pengiriman…") —
masuk sheet Perilaku Terkonfirmasi.

Tiga pengerasan selesaikan_order dari kegagalan nyata: panel notifikasi
yang menutupi app terdeteksi dan ditutup (pernah menipu jadi "order
hilang"), layar non-app dipulihkan via activate_app alih-alih Back buta
(pernah mundur sampai launcher), dan ID form di-poll dulu (konten
jaringan telat → form sah pernah dibatalkan sebagai salah kartu).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -841,7 +841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -935,12 +935,24 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Push notifikasi penugasan (FCM)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
           <t>Nol crash/ANR</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>Sepanjang seluruh run 16-17 Agu (11 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Sepanjang seluruh run 16-17 Agu (12 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
seed_ftl MULTIPICKUP + BUG-005: order multipickup tak tampil di app sopir
Seeder paham multipickup (pengirim[] ber-urutan, barang ber-pickupPartyIdx
dari template SHP26070432; droppoint kini bisa dipilih by-nama). Rantai
seed SHP26080011→FTL6941601827 sukses ASSIGNED di web — lalu uji
diferensial menemukan BUG-005 (HIGH): order MULTIPICKUP tidak pernah
muncul di daftar tugas app, padahal push FCM-nya terkirim-diterima dan
order NORMAL kembar identiknya tampil seketika. Jalur list
(GET api/v1/mobile/penugasan, apicore-staging — base mobile API
dipetakan dari DEX) tidak konsisten dengan jalur push; order multipickup
lama COMPLETED menandakan regresi. Order repro dibiarkan ASSIGNED di
staging untuk tim dev.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Info" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temuan Bug'!$A$1:$L$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Temuan Bug'!$A$1:$L$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:L6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -829,8 +829,72 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BUG-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>17/08/2026</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Backend App / API</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Order FTL MULTIPICKUP tidak muncul di daftar tugas app sopir</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Driver Hub [STG] v2.2.0-stg, Galaxy A52s (Android 14), staging</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>1. Seed dua order FTL identik (sopir/armada/PIC/rute sama), beda tipePengiriman: NORMAL vs MULTIPICKUP
+2. Penugasan keduanya ke sopir yang sama
+3. Buka app sopir, refresh berkali-kali</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Order NORMAL (FTL6940683725) tampil + push FCM; order MULTIPICKUP (FTL6941601827) TIDAK PERNAH tampil — padahal push FCM-nya terkirim &amp; diterima (dumpsys notification) dan web menandai ASSIGNED</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Semua order ter-assign tampil di daftar tugas sopir, konsisten dengan push yang dikirim</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Uji diferensial 17 Agu; order multipickup lama (FTL5469870495) COMPLETED → dulu pernah bisa (indikasi regresi). Order repro FTL6941601827 dibiarkan ASSIGNED di staging</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Periksa filter GET api/v1/mobile/penugasan (apicore-staging) untuk tipePengiriman MULTIPICKUP; sinkronkan kontrak list vs push</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L5"/>
+  <autoFilter ref="A1:L6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Multipickup kedua tuntas 6 tahap; BUG-005 direvisi jadi keterlambatan
Order multipickup kedua (SHP26080012→FTL6942920480, sopir Muhaimin)
tampil di app dan diselesaikan penuh — siklusnya muat per titik (2x
Berangkat/Selesai Muat) lalu bongkar; judul kartunya berformat
"Multipickup - <kota tujuan>". Saat itu pula order multipickup pertama
ikut muncul: BUG-005 direvisi jujur dari "tidak pernah tampil" menjadi
"terlambat ±1 jam" (push seketika, list menyusul — kemungkinan cache/
materialisasi tertunda di GET api/v1/mobile/penugasan; tetap HIGH karena
di jendela itu sopir dinotifikasi tapi tak menemukan tugasnya).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -847,7 +847,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Order FTL MULTIPICKUP tidak muncul di daftar tugas app sopir</t>
+          <t>Order FTL MULTIPICKUP terlambat tampil (±1 jam) di daftar tugas app</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -869,27 +869,27 @@
         <is>
           <t>1. Seed dua order FTL identik (sopir/armada/PIC/rute sama), beda tipePengiriman: NORMAL vs MULTIPICKUP
 2. Penugasan keduanya ke sopir yang sama
-3. Buka app sopir, refresh berkali-kali</t>
+3. Buka app sopir, refresh berkali-kali; pantau selama 1 jam</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Order NORMAL (FTL6940683725) tampil + push FCM; order MULTIPICKUP (FTL6941601827) TIDAK PERNAH tampil — padahal push FCM-nya terkirim &amp; diterima (dumpsys notification) dan web menandai ASSIGNED</t>
+          <t>NORMAL (FTL6940683725) tampil dalam hitungan detik + push FCM; MULTIPICKUP (FTL6941601827) push-nya langsung diterima tapi daftar tugas kosong ±1 jam — baru tampil bersamaan saat order multipickup kedua (FTL6942920480) dibuat</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Semua order ter-assign tampil di daftar tugas sopir, konsisten dengan push yang dikirim</t>
+          <t>Daftar tugas konsisten dengan push: order ter-assign tampil seketika, apa pun tipePengiriman-nya</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>Uji diferensial 17 Agu; order multipickup lama (FTL5469870495) COMPLETED → dulu pernah bisa (indikasi regresi). Order repro FTL6941601827 dibiarkan ASSIGNED di staging</t>
+          <t>Uji diferensial + kronologi 17 Agu; sopir &amp; PIC terverifikasi identik. Sesudah tampil, siklus multipickup normal (6 tahap, muat per titik)</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>Periksa filter GET api/v1/mobile/penugasan (apicore-staging) untuk tipePengiriman MULTIPICKUP; sinkronkan kontrak list vs push</t>
+          <t>Periksa cache/materialisasi GET api/v1/mobile/penugasan (apicore-staging) untuk MULTIPICKUP; samakan latensi list dengan push</t>
         </is>
       </c>
     </row>
@@ -905,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -999,22 +999,34 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Push notifikasi penugasan (FCM)</t>
+          <t>Siklus multipickup: muat per titik</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+          <t>Order MULTIPICKUP menjalani Berangkat/Selesai Muat SATU KALI PER titik muat (2 titik = 6 tahap total), judul kartu 'Multipickup - &lt;kota tujuan&gt;'. Terverifikasi penuh pada FTL6942920480.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
+          <t>Push notifikasi penugasan (FCM)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
           <t>Nol crash/ANR</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Sepanjang seluruh run 16-17 Agu (12 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
         </is>

</xml_diff>

<commit_message>
seed_ftl MULTIDROP tuntas: bongkar per titik + pemilih alamat di loop
Seeder paham multidrop (penerima[] ber-urutan, barang ber-dropOffPartyIdx
dari template SHP26080002; CLI ftl-<tipe> generik). Siklusnya cermin
multipickup: 1x muat lalu Berangkat/Selesai Bongkar per titik drop —
Berangkat Bongkar menuntut "Pilih Alamat" (bottom-sheet alamat drop;
validasi "Pilih alamat tujuan terlebih dahulu" masuk oracle), titik
terakhir dipilih otomatis oleh app. Loop kini membuka sheet itu dan
memilih alamat pertama; server yang menentukan giliran sah.

FTL6944366042 selesai penuh (COMPLETED di web, nol crash). Adendum
BUG-005: multidrop tampil SEKETIKA — keterlambatan spesifik multipickup
atau intermiten.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -905,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1011,22 +1011,34 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Push notifikasi penugasan (FCM)</t>
+          <t>Siklus multidrop: bongkar per titik + pemilih alamat</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+          <t>Order MULTIDROP: 1x siklus muat lalu Berangkat/Selesai Bongkar per titik drop; Berangkat Bongkar menuntut 'Pilih Alamat' (bottom-sheet alamat tiap drop; validasi 'Pilih alamat tujuan terlebih dahulu'), dan titik TERAKHIR dipilih otomatis. Judul kartu '&lt;kota asal&gt; - Multidrop'. Muncul SEKETIKA di app (keterlambatan BUG-005 tidak terjadi — spesifik multipickup/intermiten). Terverifikasi penuh pada FTL6944366042.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Push notifikasi penugasan (FCM)</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Nol crash/ANR</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Sepanjang seluruh run 16-17 Agu (12 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
         </is>

</xml_diff>

<commit_message>
seed_ftl MULTIPOINT: matriks FTL lengkap teruji end-to-end
"Multipoint" di UI = enum API MULTIDROP_MULTIPICKUP (dibocorkan pesan
validator — tidak ada template di staging, payload disusun dari
hipotesis gabungan dan lolos sekali coba: barang membawa pickupPartyIdx
DAN dropOffPartyIdx). FTL6945224841 selesai penuh 8 tahap: muat per
titik pickup lalu bongkar per titik drop dengan Pilih Alamat; tampil
seketika di app (adendum BUG-005: keterlambatan makin spesifik ke
multipickup murni). Matriks FTL tuntas: Normal, Multipickup, Multidrop,
Multipoint.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -905,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1023,22 +1023,34 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Push notifikasi penugasan (FCM)</t>
+          <t>Siklus multipoint (MULTIDROP_MULTIPICKUP)</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+          <t>Nama UI 'Multipoint' = enum API MULTIDROP_MULTIPICKUP (dibocorkan validator). Siklus = gabungan penuh: muat per titik pickup lalu bongkar per titik drop (2+2 titik = 8 tahap), judul kartu 'Multipickup - Multidrop', tampil seketika di app. Terverifikasi penuh pada FTL6945224841 — melengkapi matriks FTL: Normal/Multipickup/Multidrop/Multipoint semuanya teruji end-to-end.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
+          <t>Push notifikasi penugasan (FCM)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
           <t>Nol crash/ANR</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Sepanjang seluruh run 16-17 Agu (12 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
         </is>

</xml_diff>

<commit_message>
seed_fcl: rantai FCL Normal sampai ASSIGNED; FCL/LCL by design non-app
Kontrak laut terpetakan dari template SHP26070422 + order FCL5723465748:
shipment membawa pelabuhan+jenisKontainer+jumlahArmada, order menambah
jenisJadwal/pelayaran/namaKapal/voyage/closingTime/etd/eta (tanpa
jenisArmadaId); master /pelabuhans /jenis-kontainers /pelayarans. Unit
penugasan FCL = armada+sopir+jenisKontainerId — sopirId hanya sah
bersama armadaId (aturan validator), kontainer-saja diterima tapi tak
menjangkau siapa pun.

Konfirmasi produk: FCL/LCL tidak masuk app sopir (dikerjakan dari web),
jadi seed berhenti sah di ASSIGNED tanpa push/kartu — bukan bug; masuk
sheet Perilaku Terkonfirmasi. Dua order uji FCL ditinggal ASSIGNED di
staging.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/report/laporan_bug_2026-08-17.xlsx
+++ b/report/laporan_bug_2026-08-17.xlsx
@@ -905,7 +905,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1035,22 +1035,34 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Push notifikasi penugasan (FCM)</t>
+          <t>FCL/LCL tidak masuk app sopir (by design)</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+          <t>Konfirmasi produk 17 Agu: order moda laut dikerjakan dari web, bukan app sopir — penugasan FCL ASSIGNED memang tanpa push FCM dan tanpa kartu di HP. Seeder (seed_fcl) mendukung rantai FCL sampai ASSIGNED untuk pengujian sisi web; kontrak unit FCL: armada+sopir+jenisKontainerId (kontainer saja juga diterima validator).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Push notifikasi penugasan (FCM)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Begitu penugasan dibuat di TMS, HP sopir menerima notifikasi 'Anda menerima tugas pengiriman pada nomor order …' (terverifikasi 17 Agu pada order seed LKL-FTL6940683725).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Nol crash/ANR</t>
         </is>
       </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Sepanjang seluruh run 16-17 Agu (12 order diselesaikan end-to-end) tidak ada FATAL EXCEPTION maupun ANR di logcat aplikasi.</t>
         </is>

</xml_diff>